<commit_message>
Match Portfolio_Master format in Excel export; add Signal+CompScore to Holdings sheet; composite score rotation; rules page update
</commit_message>
<xml_diff>
--- a/Portfolio_Reports/Portfolio_Master.xlsx
+++ b/Portfolio_Reports/Portfolio_Master.xlsx
@@ -190,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="189">
+  <cellXfs count="251">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -707,6 +707,192 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1200,13 +1386,13 @@
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="105" t="inlineStr">
+      <c r="A2" s="189" t="inlineStr">
         <is>
           <t>2026-04-22</t>
         </is>
       </c>
       <c r="B2" s="55" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2" s="56" t="n">
         <v>303748.3059307933</v>
@@ -1240,82 +1426,82 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="105" t="inlineStr">
+      <c r="A3" s="189" t="inlineStr">
         <is>
           <t>2026-04-23</t>
         </is>
       </c>
-      <c r="B3" s="106" t="n">
-        <v>6</v>
-      </c>
-      <c r="C3" s="107" t="n">
+      <c r="B3" s="190" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" s="191" t="n">
         <v>299325.3084818721</v>
       </c>
-      <c r="D3" s="108" t="n">
+      <c r="D3" s="192" t="n">
         <v>29448.30848187208</v>
       </c>
-      <c r="E3" s="109" t="n">
+      <c r="E3" s="193" t="n">
         <v>269877</v>
       </c>
-      <c r="F3" s="110" t="n">
+      <c r="F3" s="194" t="n">
         <v>-674.6915181279182</v>
       </c>
-      <c r="G3" s="111" t="n">
+      <c r="G3" s="195" t="n">
         <v>-0.002248971727093061</v>
       </c>
-      <c r="H3" s="112" t="n">
+      <c r="H3" s="196" t="n">
         <v>0</v>
       </c>
-      <c r="I3" s="113" t="n">
+      <c r="I3" s="197" t="n">
         <v>-0.01456138968534346</v>
       </c>
-      <c r="J3" s="114" t="n">
+      <c r="J3" s="198" t="n">
         <v>10</v>
       </c>
-      <c r="K3" s="115" t="n">
+      <c r="K3" s="199" t="n">
         <v>0</v>
       </c>
-      <c r="L3" s="116" t="n">
+      <c r="L3" s="200" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="147" t="inlineStr">
+      <c r="A4" s="189" t="inlineStr">
         <is>
           <t>2026-04-24</t>
         </is>
       </c>
-      <c r="B4" s="148" t="n">
-        <v>7</v>
-      </c>
-      <c r="C4" s="149" t="n">
-        <v>299325.3084818721</v>
-      </c>
-      <c r="D4" s="150" t="n">
+      <c r="B4" s="190" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" s="191" t="n">
+        <v>299017.3066517711</v>
+      </c>
+      <c r="D4" s="192" t="n">
         <v>29448.30848187208</v>
       </c>
-      <c r="E4" s="151" t="n">
-        <v>269877</v>
-      </c>
-      <c r="F4" s="152" t="n">
-        <v>-674.6915181279182</v>
-      </c>
-      <c r="G4" s="153" t="n">
-        <v>-0.002248971727093061</v>
-      </c>
-      <c r="H4" s="154" t="n">
+      <c r="E4" s="193" t="n">
+        <v>269568.998169899</v>
+      </c>
+      <c r="F4" s="194" t="n">
+        <v>-982.6933482289314</v>
+      </c>
+      <c r="G4" s="195" t="n">
+        <v>-0.003275644494096438</v>
+      </c>
+      <c r="H4" s="196" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="155" t="n">
-        <v>-0.01456138968534346</v>
-      </c>
-      <c r="J4" s="156" t="n">
+      <c r="I4" s="197" t="n">
+        <v>-0.01557539313519707</v>
+      </c>
+      <c r="J4" s="198" t="n">
         <v>10</v>
       </c>
-      <c r="K4" s="157" t="n">
+      <c r="K4" s="199" t="n">
         <v>0</v>
       </c>
-      <c r="L4" s="158" t="n">
+      <c r="L4" s="200" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1346,454 +1532,454 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="159" t="inlineStr">
+      <c r="A1" s="201" t="inlineStr">
         <is>
           <t>Current Holdings  —  24 Apr 2026</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="160" t="inlineStr">
+      <c r="A2" s="202" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B2" s="160" t="inlineStr">
+      <c r="B2" s="202" t="inlineStr">
         <is>
           <t>Stock Name</t>
         </is>
       </c>
-      <c r="C2" s="160" t="inlineStr">
+      <c r="C2" s="202" t="inlineStr">
         <is>
           <t>Shares</t>
         </is>
       </c>
-      <c r="D2" s="160" t="inlineStr">
+      <c r="D2" s="202" t="inlineStr">
         <is>
           <t>Avg Cost (฿)</t>
         </is>
       </c>
-      <c r="E2" s="160" t="inlineStr">
+      <c r="E2" s="202" t="inlineStr">
         <is>
           <t>Current Price (฿)</t>
         </is>
       </c>
-      <c r="F2" s="160" t="inlineStr">
+      <c r="F2" s="202" t="inlineStr">
         <is>
           <t>Market Value (฿)</t>
         </is>
       </c>
-      <c r="G2" s="160" t="inlineStr">
+      <c r="G2" s="202" t="inlineStr">
         <is>
           <t>Unrealised P&amp;L (฿)</t>
         </is>
       </c>
-      <c r="H2" s="160" t="inlineStr">
+      <c r="H2" s="202" t="inlineStr">
         <is>
           <t>P&amp;L %</t>
         </is>
       </c>
-      <c r="I2" s="160" t="inlineStr">
+      <c r="I2" s="202" t="inlineStr">
         <is>
           <t>Entry Date</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="161" t="inlineStr">
+      <c r="A3" s="203" t="inlineStr">
+        <is>
+          <t>SIRI.BK</t>
+        </is>
+      </c>
+      <c r="B3" s="204" t="inlineStr">
+        <is>
+          <t>SIRI</t>
+        </is>
+      </c>
+      <c r="C3" s="205" t="n">
+        <v>20200</v>
+      </c>
+      <c r="D3" s="206" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="E3" s="207" t="n">
+        <v>1.409999966621399</v>
+      </c>
+      <c r="F3" s="208">
+        <f>C3*E3</f>
+        <v/>
+      </c>
+      <c r="G3" s="209">
+        <f>F3-C3*D3</f>
+        <v/>
+      </c>
+      <c r="H3" s="210">
+        <f>(E3-D3)/D3</f>
+        <v/>
+      </c>
+      <c r="I3" s="211" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="203" t="inlineStr">
+        <is>
+          <t>JASIF.BK</t>
+        </is>
+      </c>
+      <c r="B4" s="204" t="inlineStr">
+        <is>
+          <t>JASIF</t>
+        </is>
+      </c>
+      <c r="C4" s="205" t="n">
+        <v>4200</v>
+      </c>
+      <c r="D4" s="206" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="E4" s="207" t="n">
+        <v>6.699999809265137</v>
+      </c>
+      <c r="F4" s="208">
+        <f>C4*E4</f>
+        <v/>
+      </c>
+      <c r="G4" s="209">
+        <f>F4-C4*D4</f>
+        <v/>
+      </c>
+      <c r="H4" s="210">
+        <f>(E4-D4)/D4</f>
+        <v/>
+      </c>
+      <c r="I4" s="211" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="203" t="inlineStr">
+        <is>
+          <t>WHA.BK</t>
+        </is>
+      </c>
+      <c r="B5" s="204" t="inlineStr">
+        <is>
+          <t>WHA</t>
+        </is>
+      </c>
+      <c r="C5" s="205" t="n">
+        <v>6400</v>
+      </c>
+      <c r="D5" s="206" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="E5" s="207" t="n">
+        <v>4.380000114440918</v>
+      </c>
+      <c r="F5" s="208">
+        <f>C5*E5</f>
+        <v/>
+      </c>
+      <c r="G5" s="209">
+        <f>F5-C5*D5</f>
+        <v/>
+      </c>
+      <c r="H5" s="210">
+        <f>(E5-D5)/D5</f>
+        <v/>
+      </c>
+      <c r="I5" s="211" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="203" t="inlineStr">
         <is>
           <t>TU.BK</t>
         </is>
       </c>
-      <c r="B3" s="162" t="inlineStr">
+      <c r="B6" s="204" t="inlineStr">
         <is>
           <t>TU</t>
         </is>
       </c>
-      <c r="C3" s="163" t="n">
+      <c r="C6" s="205" t="n">
         <v>2500</v>
       </c>
-      <c r="D3" s="164" t="n">
+      <c r="D6" s="206" t="n">
         <v>11.4</v>
       </c>
-      <c r="E3" s="165" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="F3" s="166">
-        <f>C3*E3</f>
-        <v/>
-      </c>
-      <c r="G3" s="167">
-        <f>F3-C3*D3</f>
-        <v/>
-      </c>
-      <c r="H3" s="168">
-        <f>(E3-D3)/D3</f>
-        <v/>
-      </c>
-      <c r="I3" s="169" t="inlineStr">
+      <c r="E6" s="207" t="n">
+        <v>11.19999980926514</v>
+      </c>
+      <c r="F6" s="208">
+        <f>C6*E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="209">
+        <f>F6-C6*D6</f>
+        <v/>
+      </c>
+      <c r="H6" s="210">
+        <f>(E6-D6)/D6</f>
+        <v/>
+      </c>
+      <c r="I6" s="211" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="161" t="inlineStr">
-        <is>
-          <t>SIRI.BK</t>
-        </is>
-      </c>
-      <c r="B4" s="162" t="inlineStr">
-        <is>
-          <t>SIRI</t>
-        </is>
-      </c>
-      <c r="C4" s="163" t="n">
-        <v>20200</v>
-      </c>
-      <c r="D4" s="164" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="E4" s="165" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="F4" s="166">
-        <f>C4*E4</f>
-        <v/>
-      </c>
-      <c r="G4" s="167">
-        <f>F4-C4*D4</f>
-        <v/>
-      </c>
-      <c r="H4" s="168">
-        <f>(E4-D4)/D4</f>
-        <v/>
-      </c>
-      <c r="I4" s="169" t="inlineStr">
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="212" t="inlineStr">
+        <is>
+          <t>TQM.BK</t>
+        </is>
+      </c>
+      <c r="B7" s="213" t="inlineStr">
+        <is>
+          <t>TQM</t>
+        </is>
+      </c>
+      <c r="C7" s="214" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D7" s="215" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="E7" s="216" t="n">
+        <v>13.80000019073486</v>
+      </c>
+      <c r="F7" s="217">
+        <f>C7*E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="218">
+        <f>F7-C7*D7</f>
+        <v/>
+      </c>
+      <c r="H7" s="219">
+        <f>(E7-D7)/D7</f>
+        <v/>
+      </c>
+      <c r="I7" s="220" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="161" t="inlineStr">
-        <is>
-          <t>WHA.BK</t>
-        </is>
-      </c>
-      <c r="B5" s="162" t="inlineStr">
-        <is>
-          <t>WHA</t>
-        </is>
-      </c>
-      <c r="C5" s="163" t="n">
-        <v>6400</v>
-      </c>
-      <c r="D5" s="164" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="E5" s="165" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F5" s="166">
-        <f>C5*E5</f>
-        <v/>
-      </c>
-      <c r="G5" s="167">
-        <f>F5-C5*D5</f>
-        <v/>
-      </c>
-      <c r="H5" s="168">
-        <f>(E5-D5)/D5</f>
-        <v/>
-      </c>
-      <c r="I5" s="169" t="inlineStr">
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="212" t="inlineStr">
+        <is>
+          <t>BAY.BK</t>
+        </is>
+      </c>
+      <c r="B8" s="213" t="inlineStr">
+        <is>
+          <t>BAY</t>
+        </is>
+      </c>
+      <c r="C8" s="214" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D8" s="215" t="n">
+        <v>26</v>
+      </c>
+      <c r="E8" s="216" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="F8" s="217">
+        <f>C8*E8</f>
+        <v/>
+      </c>
+      <c r="G8" s="218">
+        <f>F8-C8*D8</f>
+        <v/>
+      </c>
+      <c r="H8" s="219">
+        <f>(E8-D8)/D8</f>
+        <v/>
+      </c>
+      <c r="I8" s="220" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="161" t="inlineStr">
-        <is>
-          <t>JASIF.BK</t>
-        </is>
-      </c>
-      <c r="B6" s="162" t="inlineStr">
-        <is>
-          <t>JASIF</t>
-        </is>
-      </c>
-      <c r="C6" s="163" t="n">
-        <v>4200</v>
-      </c>
-      <c r="D6" s="164" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="E6" s="165" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="F6" s="166">
-        <f>C6*E6</f>
-        <v/>
-      </c>
-      <c r="G6" s="167">
-        <f>F6-C6*D6</f>
-        <v/>
-      </c>
-      <c r="H6" s="168">
-        <f>(E6-D6)/D6</f>
-        <v/>
-      </c>
-      <c r="I6" s="169" t="inlineStr">
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="221" t="inlineStr">
+        <is>
+          <t>CK.BK</t>
+        </is>
+      </c>
+      <c r="B9" s="222" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="C9" s="223" t="n">
+        <v>1600</v>
+      </c>
+      <c r="D9" s="224" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="E9" s="225" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="F9" s="226">
+        <f>C9*E9</f>
+        <v/>
+      </c>
+      <c r="G9" s="227">
+        <f>F9-C9*D9</f>
+        <v/>
+      </c>
+      <c r="H9" s="228">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="I9" s="229" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="161" t="inlineStr">
-        <is>
-          <t>CK.BK</t>
-        </is>
-      </c>
-      <c r="B7" s="162" t="inlineStr">
-        <is>
-          <t>CK</t>
-        </is>
-      </c>
-      <c r="C7" s="163" t="n">
-        <v>1600</v>
-      </c>
-      <c r="D7" s="164" t="n">
-        <v>17.2</v>
-      </c>
-      <c r="E7" s="165" t="n">
-        <v>17.2</v>
-      </c>
-      <c r="F7" s="166">
-        <f>C7*E7</f>
-        <v/>
-      </c>
-      <c r="G7" s="167">
-        <f>F7-C7*D7</f>
-        <v/>
-      </c>
-      <c r="H7" s="168">
-        <f>(E7-D7)/D7</f>
-        <v/>
-      </c>
-      <c r="I7" s="169" t="inlineStr">
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="203" t="inlineStr">
+        <is>
+          <t>AMATA.BK</t>
+        </is>
+      </c>
+      <c r="B10" s="204" t="inlineStr">
+        <is>
+          <t>AMATA</t>
+        </is>
+      </c>
+      <c r="C10" s="205" t="n">
+        <v>1300</v>
+      </c>
+      <c r="D10" s="206" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="E10" s="207" t="n">
+        <v>20.29999923706055</v>
+      </c>
+      <c r="F10" s="208">
+        <f>C10*E10</f>
+        <v/>
+      </c>
+      <c r="G10" s="209">
+        <f>F10-C10*D10</f>
+        <v/>
+      </c>
+      <c r="H10" s="210">
+        <f>(E10-D10)/D10</f>
+        <v/>
+      </c>
+      <c r="I10" s="211" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="161" t="inlineStr">
-        <is>
-          <t>TQM.BK</t>
-        </is>
-      </c>
-      <c r="B8" s="162" t="inlineStr">
-        <is>
-          <t>TQM</t>
-        </is>
-      </c>
-      <c r="C8" s="163" t="n">
-        <v>2000</v>
-      </c>
-      <c r="D8" s="164" t="n">
-        <v>13.7</v>
-      </c>
-      <c r="E8" s="165" t="n">
-        <v>13.7</v>
-      </c>
-      <c r="F8" s="166">
-        <f>C8*E8</f>
-        <v/>
-      </c>
-      <c r="G8" s="167">
-        <f>F8-C8*D8</f>
-        <v/>
-      </c>
-      <c r="H8" s="168">
-        <f>(E8-D8)/D8</f>
-        <v/>
-      </c>
-      <c r="I8" s="169" t="inlineStr">
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="203" t="inlineStr">
+        <is>
+          <t>KTC.BK</t>
+        </is>
+      </c>
+      <c r="B11" s="204" t="inlineStr">
+        <is>
+          <t>KTC</t>
+        </is>
+      </c>
+      <c r="C11" s="205" t="n">
+        <v>900</v>
+      </c>
+      <c r="D11" s="206" t="n">
+        <v>29.25</v>
+      </c>
+      <c r="E11" s="207" t="n">
+        <v>29.25</v>
+      </c>
+      <c r="F11" s="208">
+        <f>C11*E11</f>
+        <v/>
+      </c>
+      <c r="G11" s="230">
+        <f>F11-C11*D11</f>
+        <v/>
+      </c>
+      <c r="H11" s="231">
+        <f>(E11-D11)/D11</f>
+        <v/>
+      </c>
+      <c r="I11" s="211" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="161" t="inlineStr">
-        <is>
-          <t>AMATA.BK</t>
-        </is>
-      </c>
-      <c r="B9" s="162" t="inlineStr">
-        <is>
-          <t>AMATA</t>
-        </is>
-      </c>
-      <c r="C9" s="163" t="n">
-        <v>1300</v>
-      </c>
-      <c r="D9" s="164" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="E9" s="165" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="F9" s="166">
-        <f>C9*E9</f>
-        <v/>
-      </c>
-      <c r="G9" s="167">
-        <f>F9-C9*D9</f>
-        <v/>
-      </c>
-      <c r="H9" s="168">
-        <f>(E9-D9)/D9</f>
-        <v/>
-      </c>
-      <c r="I9" s="169" t="inlineStr">
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="203" t="inlineStr">
+        <is>
+          <t>TISCO.BK</t>
+        </is>
+      </c>
+      <c r="B12" s="204" t="inlineStr">
+        <is>
+          <t>TISCO</t>
+        </is>
+      </c>
+      <c r="C12" s="205" t="n">
+        <v>200</v>
+      </c>
+      <c r="D12" s="206" t="n">
+        <v>113.5</v>
+      </c>
+      <c r="E12" s="207" t="n">
+        <v>113.5</v>
+      </c>
+      <c r="F12" s="208">
+        <f>C12*E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="230">
+        <f>F12-C12*D12</f>
+        <v/>
+      </c>
+      <c r="H12" s="231">
+        <f>(E12-D12)/D12</f>
+        <v/>
+      </c>
+      <c r="I12" s="211" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="161" t="inlineStr">
-        <is>
-          <t>KTC.BK</t>
-        </is>
-      </c>
-      <c r="B10" s="162" t="inlineStr">
-        <is>
-          <t>KTC</t>
-        </is>
-      </c>
-      <c r="C10" s="163" t="n">
-        <v>900</v>
-      </c>
-      <c r="D10" s="164" t="n">
-        <v>29.25</v>
-      </c>
-      <c r="E10" s="165" t="n">
-        <v>29.25</v>
-      </c>
-      <c r="F10" s="166">
-        <f>C10*E10</f>
-        <v/>
-      </c>
-      <c r="G10" s="167">
-        <f>F10-C10*D10</f>
-        <v/>
-      </c>
-      <c r="H10" s="168">
-        <f>(E10-D10)/D10</f>
-        <v/>
-      </c>
-      <c r="I10" s="169" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="161" t="inlineStr">
-        <is>
-          <t>BAY.BK</t>
-        </is>
-      </c>
-      <c r="B11" s="162" t="inlineStr">
-        <is>
-          <t>BAY</t>
-        </is>
-      </c>
-      <c r="C11" s="163" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D11" s="164" t="n">
-        <v>26</v>
-      </c>
-      <c r="E11" s="165" t="n">
-        <v>26</v>
-      </c>
-      <c r="F11" s="166">
-        <f>C11*E11</f>
-        <v/>
-      </c>
-      <c r="G11" s="167">
-        <f>F11-C11*D11</f>
-        <v/>
-      </c>
-      <c r="H11" s="168">
-        <f>(E11-D11)/D11</f>
-        <v/>
-      </c>
-      <c r="I11" s="169" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="161" t="inlineStr">
-        <is>
-          <t>TISCO.BK</t>
-        </is>
-      </c>
-      <c r="B12" s="162" t="inlineStr">
-        <is>
-          <t>TISCO</t>
-        </is>
-      </c>
-      <c r="C12" s="163" t="n">
-        <v>200</v>
-      </c>
-      <c r="D12" s="164" t="n">
-        <v>113.5</v>
-      </c>
-      <c r="E12" s="165" t="n">
-        <v>113.5</v>
-      </c>
-      <c r="F12" s="166">
-        <f>C12*E12</f>
-        <v/>
-      </c>
-      <c r="G12" s="167">
-        <f>F12-C12*D12</f>
-        <v/>
-      </c>
-      <c r="H12" s="168">
-        <f>(E12-D12)/D12</f>
-        <v/>
-      </c>
-      <c r="I12" s="169" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-    </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="170" t="inlineStr">
+      <c r="B13" s="232" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F13" s="171">
+      <c r="F13" s="233">
         <f>SUM(F3:F12)</f>
         <v/>
       </c>
-      <c r="G13" s="172">
+      <c r="G13" s="234">
         <f>SUM(G3:G12)</f>
         <v/>
       </c>
-      <c r="H13" s="173">
+      <c r="H13" s="235">
         <f>G13/SUMPRODUCT(C3:C12,D3:D12)</f>
         <v/>
       </c>
@@ -1828,14 +2014,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="159" t="inlineStr">
+      <c r="A1" s="201" t="inlineStr">
         <is>
           <t>Today's Trades  —  24 Apr 2026</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="174" t="inlineStr">
+      <c r="A3" s="236" t="inlineStr">
         <is>
           <t>No trades were executed today.</t>
         </is>
@@ -1873,509 +2059,509 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="159" t="inlineStr">
+      <c r="A1" s="201" t="inlineStr">
         <is>
           <t>Complete Trade History  —  since 2026-04-21</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="160" t="inlineStr">
+      <c r="A2" s="202" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B2" s="160" t="inlineStr">
+      <c r="B2" s="202" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="C2" s="160" t="inlineStr">
+      <c r="C2" s="202" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="D2" s="160" t="inlineStr">
+      <c r="D2" s="202" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="E2" s="160" t="inlineStr">
+      <c r="E2" s="202" t="inlineStr">
         <is>
           <t>Shares</t>
         </is>
       </c>
-      <c r="F2" s="160" t="inlineStr">
+      <c r="F2" s="202" t="inlineStr">
         <is>
           <t>Price (฿)</t>
         </is>
       </c>
-      <c r="G2" s="160" t="inlineStr">
+      <c r="G2" s="202" t="inlineStr">
         <is>
           <t>Lots</t>
         </is>
       </c>
-      <c r="H2" s="160" t="inlineStr">
+      <c r="H2" s="202" t="inlineStr">
         <is>
           <t>Value (฿)</t>
         </is>
       </c>
-      <c r="I2" s="160" t="inlineStr">
+      <c r="I2" s="202" t="inlineStr">
         <is>
           <t>Realised P&amp;L (฿)</t>
         </is>
       </c>
-      <c r="J2" s="160" t="inlineStr">
+      <c r="J2" s="202" t="inlineStr">
         <is>
           <t>Reason / Signal</t>
         </is>
       </c>
     </row>
     <row r="3" ht="17" customHeight="1">
-      <c r="A3" s="175" t="inlineStr">
+      <c r="A3" s="237" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B3" s="176" t="inlineStr">
+      <c r="B3" s="238" t="inlineStr">
         <is>
           <t>TISCO.BK</t>
         </is>
       </c>
-      <c r="C3" s="177" t="inlineStr">
+      <c r="C3" s="239" t="inlineStr">
         <is>
           <t>TISCO</t>
         </is>
       </c>
-      <c r="D3" s="178" t="inlineStr">
+      <c r="D3" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E3" s="179" t="n">
+      <c r="E3" s="241" t="n">
         <v>200</v>
       </c>
-      <c r="F3" s="180" t="n">
+      <c r="F3" s="242" t="n">
         <v>113.5</v>
       </c>
-      <c r="G3" s="179" t="n">
+      <c r="G3" s="241" t="n">
         <v>2</v>
       </c>
-      <c r="H3" s="181">
+      <c r="H3" s="243">
         <f>E3*F3</f>
         <v/>
       </c>
-      <c r="I3" s="182" t="inlineStr">
+      <c r="I3" s="244" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J3" s="183" t="inlineStr">
+      <c r="J3" s="245" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="17" customHeight="1">
-      <c r="A4" s="184" t="inlineStr">
+      <c r="A4" s="246" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B4" s="185" t="inlineStr">
+      <c r="B4" s="247" t="inlineStr">
         <is>
           <t>SIRI.BK</t>
         </is>
       </c>
-      <c r="C4" s="162" t="inlineStr">
+      <c r="C4" s="204" t="inlineStr">
         <is>
           <t>SIRI</t>
         </is>
       </c>
-      <c r="D4" s="178" t="inlineStr">
+      <c r="D4" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E4" s="163" t="n">
+      <c r="E4" s="205" t="n">
         <v>20200</v>
       </c>
-      <c r="F4" s="164" t="n">
+      <c r="F4" s="206" t="n">
         <v>1.41</v>
       </c>
-      <c r="G4" s="163" t="n">
+      <c r="G4" s="205" t="n">
         <v>202</v>
       </c>
-      <c r="H4" s="166">
+      <c r="H4" s="208">
         <f>E4*F4</f>
         <v/>
       </c>
-      <c r="I4" s="186" t="inlineStr">
+      <c r="I4" s="248" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J4" s="187" t="inlineStr">
+      <c r="J4" s="249" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="175" t="inlineStr">
+      <c r="A5" s="237" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B5" s="176" t="inlineStr">
+      <c r="B5" s="238" t="inlineStr">
         <is>
           <t>TU.BK</t>
         </is>
       </c>
-      <c r="C5" s="177" t="inlineStr">
+      <c r="C5" s="239" t="inlineStr">
         <is>
           <t>TU</t>
         </is>
       </c>
-      <c r="D5" s="178" t="inlineStr">
+      <c r="D5" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E5" s="179" t="n">
+      <c r="E5" s="241" t="n">
         <v>2500</v>
       </c>
-      <c r="F5" s="180" t="n">
+      <c r="F5" s="242" t="n">
         <v>11.4</v>
       </c>
-      <c r="G5" s="179" t="n">
+      <c r="G5" s="241" t="n">
         <v>25</v>
       </c>
-      <c r="H5" s="181">
+      <c r="H5" s="243">
         <f>E5*F5</f>
         <v/>
       </c>
-      <c r="I5" s="182" t="inlineStr">
+      <c r="I5" s="244" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J5" s="183" t="inlineStr">
+      <c r="J5" s="245" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="184" t="inlineStr">
+      <c r="A6" s="246" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B6" s="185" t="inlineStr">
+      <c r="B6" s="247" t="inlineStr">
         <is>
           <t>BAY.BK</t>
         </is>
       </c>
-      <c r="C6" s="162" t="inlineStr">
+      <c r="C6" s="204" t="inlineStr">
         <is>
           <t>BAY</t>
         </is>
       </c>
-      <c r="D6" s="178" t="inlineStr">
+      <c r="D6" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E6" s="163" t="n">
+      <c r="E6" s="205" t="n">
         <v>1000</v>
       </c>
-      <c r="F6" s="164" t="n">
+      <c r="F6" s="206" t="n">
         <v>26</v>
       </c>
-      <c r="G6" s="163" t="n">
+      <c r="G6" s="205" t="n">
         <v>10</v>
       </c>
-      <c r="H6" s="166">
+      <c r="H6" s="208">
         <f>E6*F6</f>
         <v/>
       </c>
-      <c r="I6" s="186" t="inlineStr">
+      <c r="I6" s="248" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J6" s="187" t="inlineStr">
+      <c r="J6" s="249" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="175" t="inlineStr">
+      <c r="A7" s="237" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B7" s="176" t="inlineStr">
+      <c r="B7" s="238" t="inlineStr">
         <is>
           <t>KTC.BK</t>
         </is>
       </c>
-      <c r="C7" s="177" t="inlineStr">
+      <c r="C7" s="239" t="inlineStr">
         <is>
           <t>KTC</t>
         </is>
       </c>
-      <c r="D7" s="178" t="inlineStr">
+      <c r="D7" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E7" s="179" t="n">
+      <c r="E7" s="241" t="n">
         <v>900</v>
       </c>
-      <c r="F7" s="180" t="n">
+      <c r="F7" s="242" t="n">
         <v>29.25</v>
       </c>
-      <c r="G7" s="179" t="n">
+      <c r="G7" s="241" t="n">
         <v>9</v>
       </c>
-      <c r="H7" s="181">
+      <c r="H7" s="243">
         <f>E7*F7</f>
         <v/>
       </c>
-      <c r="I7" s="182" t="inlineStr">
+      <c r="I7" s="244" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J7" s="183" t="inlineStr">
+      <c r="J7" s="245" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="184" t="inlineStr">
+      <c r="A8" s="246" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B8" s="185" t="inlineStr">
+      <c r="B8" s="247" t="inlineStr">
         <is>
           <t>TQM.BK</t>
         </is>
       </c>
-      <c r="C8" s="162" t="inlineStr">
+      <c r="C8" s="204" t="inlineStr">
         <is>
           <t>TQM</t>
         </is>
       </c>
-      <c r="D8" s="178" t="inlineStr">
+      <c r="D8" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E8" s="163" t="n">
+      <c r="E8" s="205" t="n">
         <v>2000</v>
       </c>
-      <c r="F8" s="164" t="n">
+      <c r="F8" s="206" t="n">
         <v>13.7</v>
       </c>
-      <c r="G8" s="163" t="n">
+      <c r="G8" s="205" t="n">
         <v>20</v>
       </c>
-      <c r="H8" s="166">
+      <c r="H8" s="208">
         <f>E8*F8</f>
         <v/>
       </c>
-      <c r="I8" s="186" t="inlineStr">
+      <c r="I8" s="248" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J8" s="187" t="inlineStr">
+      <c r="J8" s="249" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="175" t="inlineStr">
+      <c r="A9" s="237" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B9" s="176" t="inlineStr">
+      <c r="B9" s="238" t="inlineStr">
         <is>
           <t>WHA.BK</t>
         </is>
       </c>
-      <c r="C9" s="177" t="inlineStr">
+      <c r="C9" s="239" t="inlineStr">
         <is>
           <t>WHA</t>
         </is>
       </c>
-      <c r="D9" s="178" t="inlineStr">
+      <c r="D9" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E9" s="179" t="n">
+      <c r="E9" s="241" t="n">
         <v>6400</v>
       </c>
-      <c r="F9" s="180" t="n">
+      <c r="F9" s="242" t="n">
         <v>4.4</v>
       </c>
-      <c r="G9" s="179" t="n">
+      <c r="G9" s="241" t="n">
         <v>64</v>
       </c>
-      <c r="H9" s="181">
+      <c r="H9" s="243">
         <f>E9*F9</f>
         <v/>
       </c>
-      <c r="I9" s="182" t="inlineStr">
+      <c r="I9" s="244" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J9" s="183" t="inlineStr">
+      <c r="J9" s="245" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="184" t="inlineStr">
+      <c r="A10" s="246" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B10" s="185" t="inlineStr">
+      <c r="B10" s="247" t="inlineStr">
         <is>
           <t>JASIF.BK</t>
         </is>
       </c>
-      <c r="C10" s="162" t="inlineStr">
+      <c r="C10" s="204" t="inlineStr">
         <is>
           <t>JASIF</t>
         </is>
       </c>
-      <c r="D10" s="178" t="inlineStr">
+      <c r="D10" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E10" s="163" t="n">
+      <c r="E10" s="205" t="n">
         <v>4200</v>
       </c>
-      <c r="F10" s="164" t="n">
+      <c r="F10" s="206" t="n">
         <v>6.7</v>
       </c>
-      <c r="G10" s="163" t="n">
+      <c r="G10" s="205" t="n">
         <v>42</v>
       </c>
-      <c r="H10" s="166">
+      <c r="H10" s="208">
         <f>E10*F10</f>
         <v/>
       </c>
-      <c r="I10" s="186" t="inlineStr">
+      <c r="I10" s="248" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J10" s="187" t="inlineStr">
+      <c r="J10" s="249" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="175" t="inlineStr">
+      <c r="A11" s="237" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B11" s="176" t="inlineStr">
+      <c r="B11" s="238" t="inlineStr">
         <is>
           <t>CK.BK</t>
         </is>
       </c>
-      <c r="C11" s="177" t="inlineStr">
+      <c r="C11" s="239" t="inlineStr">
         <is>
           <t>CK</t>
         </is>
       </c>
-      <c r="D11" s="178" t="inlineStr">
+      <c r="D11" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E11" s="179" t="n">
+      <c r="E11" s="241" t="n">
         <v>1600</v>
       </c>
-      <c r="F11" s="180" t="n">
+      <c r="F11" s="242" t="n">
         <v>17.2</v>
       </c>
-      <c r="G11" s="179" t="n">
+      <c r="G11" s="241" t="n">
         <v>16</v>
       </c>
-      <c r="H11" s="181">
+      <c r="H11" s="243">
         <f>E11*F11</f>
         <v/>
       </c>
-      <c r="I11" s="182" t="inlineStr">
+      <c r="I11" s="244" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J11" s="183" t="inlineStr">
+      <c r="J11" s="245" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="184" t="inlineStr">
+      <c r="A12" s="246" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B12" s="185" t="inlineStr">
+      <c r="B12" s="247" t="inlineStr">
         <is>
           <t>AMATA.BK</t>
         </is>
       </c>
-      <c r="C12" s="162" t="inlineStr">
+      <c r="C12" s="204" t="inlineStr">
         <is>
           <t>AMATA</t>
         </is>
       </c>
-      <c r="D12" s="178" t="inlineStr">
+      <c r="D12" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E12" s="163" t="n">
+      <c r="E12" s="205" t="n">
         <v>1300</v>
       </c>
-      <c r="F12" s="164" t="n">
+      <c r="F12" s="206" t="n">
         <v>20.5</v>
       </c>
-      <c r="G12" s="163" t="n">
+      <c r="G12" s="205" t="n">
         <v>13</v>
       </c>
-      <c r="H12" s="166">
+      <c r="H12" s="208">
         <f>E12*F12</f>
         <v/>
       </c>
-      <c r="I12" s="186" t="inlineStr">
+      <c r="I12" s="248" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J12" s="187" t="inlineStr">
+      <c r="J12" s="249" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
@@ -2387,11 +2573,11 @@
           <t>TOTAL TRADES</t>
         </is>
       </c>
-      <c r="H14" s="188">
+      <c r="H14" s="250">
         <f>SUM(H3:H12)</f>
         <v/>
       </c>
-      <c r="I14" s="188">
+      <c r="I14" s="250">
         <f>SUM(I3:I12)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
DCA update: 15 slots, 50k cap, topup script, dashboard refresh
</commit_message>
<xml_diff>
--- a/Portfolio_Reports/Portfolio_Master.xlsx
+++ b/Portfolio_Reports/Portfolio_Master.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Daily Performance" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Holdings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Today's Trades" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Trade History" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Performance" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Holdings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Today's Trades" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade History" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +27,7 @@
     <numFmt numFmtId="168" formatCode="฿#,##0;(฿#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="169" formatCode="0.00%;(0.00%);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -125,12 +125,6 @@
       <color rgb="0000B050"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFC000"/>
-      <sz val="10"/>
-    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -196,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="321">
+  <cellXfs count="251">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -881,216 +875,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1522,7 +1306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1721,46 +1505,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="251" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-      <c r="B5" s="252" t="n">
-        <v>6</v>
-      </c>
-      <c r="C5" s="253" t="n">
-        <v>299017.3066517711</v>
-      </c>
-      <c r="D5" s="254" t="n">
-        <v>29448.30848187208</v>
-      </c>
-      <c r="E5" s="255" t="n">
-        <v>269568.998169899</v>
-      </c>
-      <c r="F5" s="256" t="n">
-        <v>-982.6933482289314</v>
-      </c>
-      <c r="G5" s="257" t="n">
-        <v>-0.003275644494096438</v>
-      </c>
-      <c r="H5" s="258" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="259" t="n">
-        <v>-0.01557539313519707</v>
-      </c>
-      <c r="J5" s="260" t="n">
-        <v>10</v>
-      </c>
-      <c r="K5" s="261" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="262" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1773,7 +1517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1785,556 +1529,464 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="263" t="inlineStr">
-        <is>
-          <t>Current Holdings  —  27 Apr 2026</t>
+      <c r="A1" s="201" t="inlineStr">
+        <is>
+          <t>Current Holdings  —  24 Apr 2026</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="264" t="inlineStr">
+      <c r="A2" s="202" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B2" s="264" t="inlineStr">
+      <c r="B2" s="202" t="inlineStr">
         <is>
           <t>Stock Name</t>
         </is>
       </c>
-      <c r="C2" s="264" t="inlineStr">
+      <c r="C2" s="202" t="inlineStr">
         <is>
           <t>Shares</t>
         </is>
       </c>
-      <c r="D2" s="264" t="inlineStr">
+      <c r="D2" s="202" t="inlineStr">
         <is>
           <t>Avg Cost (฿)</t>
         </is>
       </c>
-      <c r="E2" s="264" t="inlineStr">
+      <c r="E2" s="202" t="inlineStr">
         <is>
           <t>Current Price (฿)</t>
         </is>
       </c>
-      <c r="F2" s="264" t="inlineStr">
+      <c r="F2" s="202" t="inlineStr">
         <is>
           <t>Market Value (฿)</t>
         </is>
       </c>
-      <c r="G2" s="264" t="inlineStr">
+      <c r="G2" s="202" t="inlineStr">
         <is>
           <t>Unrealised P&amp;L (฿)</t>
         </is>
       </c>
-      <c r="H2" s="264" t="inlineStr">
+      <c r="H2" s="202" t="inlineStr">
         <is>
           <t>P&amp;L %</t>
         </is>
       </c>
-      <c r="I2" s="264" t="inlineStr">
+      <c r="I2" s="202" t="inlineStr">
         <is>
           <t>Entry Date</t>
         </is>
       </c>
-      <c r="J2" s="264" t="inlineStr">
-        <is>
-          <t>Comp Score</t>
-        </is>
-      </c>
-      <c r="K2" s="264" t="inlineStr">
-        <is>
-          <t>Signal</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="265" t="inlineStr">
+      <c r="A3" s="203" t="inlineStr">
         <is>
           <t>SIRI.BK</t>
         </is>
       </c>
-      <c r="B3" s="266" t="inlineStr">
+      <c r="B3" s="204" t="inlineStr">
         <is>
           <t>SIRI</t>
         </is>
       </c>
-      <c r="C3" s="267" t="n">
+      <c r="C3" s="205" t="n">
         <v>20200</v>
       </c>
-      <c r="D3" s="268" t="n">
+      <c r="D3" s="206" t="n">
         <v>1.41</v>
       </c>
-      <c r="E3" s="269" t="n">
+      <c r="E3" s="207" t="n">
         <v>1.409999966621399</v>
       </c>
-      <c r="F3" s="270">
+      <c r="F3" s="208">
         <f>C3*E3</f>
         <v/>
       </c>
-      <c r="G3" s="271">
+      <c r="G3" s="209">
         <f>F3-C3*D3</f>
         <v/>
       </c>
-      <c r="H3" s="272">
+      <c r="H3" s="210">
         <f>(E3-D3)/D3</f>
         <v/>
       </c>
-      <c r="I3" s="273" t="inlineStr">
+      <c r="I3" s="211" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="J3" s="274" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="K3" s="275" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="265" t="inlineStr">
+      <c r="A4" s="203" t="inlineStr">
         <is>
           <t>JASIF.BK</t>
         </is>
       </c>
-      <c r="B4" s="266" t="inlineStr">
+      <c r="B4" s="204" t="inlineStr">
         <is>
           <t>JASIF</t>
         </is>
       </c>
-      <c r="C4" s="267" t="n">
+      <c r="C4" s="205" t="n">
         <v>4200</v>
       </c>
-      <c r="D4" s="268" t="n">
+      <c r="D4" s="206" t="n">
         <v>6.7</v>
       </c>
-      <c r="E4" s="269" t="n">
+      <c r="E4" s="207" t="n">
         <v>6.699999809265137</v>
       </c>
-      <c r="F4" s="270">
+      <c r="F4" s="208">
         <f>C4*E4</f>
         <v/>
       </c>
-      <c r="G4" s="271">
+      <c r="G4" s="209">
         <f>F4-C4*D4</f>
         <v/>
       </c>
-      <c r="H4" s="272">
+      <c r="H4" s="210">
         <f>(E4-D4)/D4</f>
         <v/>
       </c>
-      <c r="I4" s="273" t="inlineStr">
+      <c r="I4" s="211" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="J4" s="276" t="n">
-        <v>6.84</v>
-      </c>
-      <c r="K4" s="277" t="inlineStr">
-        <is>
-          <t>WEAK</t>
-        </is>
-      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="265" t="inlineStr">
+      <c r="A5" s="203" t="inlineStr">
         <is>
           <t>WHA.BK</t>
         </is>
       </c>
-      <c r="B5" s="266" t="inlineStr">
+      <c r="B5" s="204" t="inlineStr">
         <is>
           <t>WHA</t>
         </is>
       </c>
-      <c r="C5" s="267" t="n">
+      <c r="C5" s="205" t="n">
         <v>6400</v>
       </c>
-      <c r="D5" s="268" t="n">
+      <c r="D5" s="206" t="n">
         <v>4.4</v>
       </c>
-      <c r="E5" s="269" t="n">
+      <c r="E5" s="207" t="n">
         <v>4.380000114440918</v>
       </c>
-      <c r="F5" s="270">
+      <c r="F5" s="208">
         <f>C5*E5</f>
         <v/>
       </c>
-      <c r="G5" s="271">
+      <c r="G5" s="209">
         <f>F5-C5*D5</f>
         <v/>
       </c>
-      <c r="H5" s="272">
+      <c r="H5" s="210">
         <f>(E5-D5)/D5</f>
         <v/>
       </c>
-      <c r="I5" s="273" t="inlineStr">
+      <c r="I5" s="211" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="J5" s="276" t="n">
-        <v>7.48</v>
-      </c>
-      <c r="K5" s="277" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="265" t="inlineStr">
+      <c r="A6" s="203" t="inlineStr">
         <is>
           <t>TU.BK</t>
         </is>
       </c>
-      <c r="B6" s="266" t="inlineStr">
+      <c r="B6" s="204" t="inlineStr">
         <is>
           <t>TU</t>
         </is>
       </c>
-      <c r="C6" s="267" t="n">
+      <c r="C6" s="205" t="n">
         <v>2500</v>
       </c>
-      <c r="D6" s="268" t="n">
+      <c r="D6" s="206" t="n">
         <v>11.4</v>
       </c>
-      <c r="E6" s="269" t="n">
+      <c r="E6" s="207" t="n">
         <v>11.19999980926514</v>
       </c>
-      <c r="F6" s="270">
+      <c r="F6" s="208">
         <f>C6*E6</f>
         <v/>
       </c>
-      <c r="G6" s="271">
+      <c r="G6" s="209">
         <f>F6-C6*D6</f>
         <v/>
       </c>
-      <c r="H6" s="272">
+      <c r="H6" s="210">
         <f>(E6-D6)/D6</f>
         <v/>
       </c>
-      <c r="I6" s="273" t="inlineStr">
+      <c r="I6" s="211" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="J6" s="274" t="n">
-        <v>8.08</v>
-      </c>
-      <c r="K6" s="275" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="278" t="inlineStr">
+      <c r="A7" s="212" t="inlineStr">
         <is>
           <t>TQM.BK</t>
         </is>
       </c>
-      <c r="B7" s="279" t="inlineStr">
+      <c r="B7" s="213" t="inlineStr">
         <is>
           <t>TQM</t>
         </is>
       </c>
-      <c r="C7" s="280" t="n">
+      <c r="C7" s="214" t="n">
         <v>2000</v>
       </c>
-      <c r="D7" s="281" t="n">
+      <c r="D7" s="215" t="n">
         <v>13.7</v>
       </c>
-      <c r="E7" s="282" t="n">
+      <c r="E7" s="216" t="n">
         <v>13.80000019073486</v>
       </c>
-      <c r="F7" s="283">
+      <c r="F7" s="217">
         <f>C7*E7</f>
         <v/>
       </c>
-      <c r="G7" s="284">
+      <c r="G7" s="218">
         <f>F7-C7*D7</f>
         <v/>
       </c>
-      <c r="H7" s="285">
+      <c r="H7" s="219">
         <f>(E7-D7)/D7</f>
         <v/>
       </c>
-      <c r="I7" s="286" t="inlineStr">
+      <c r="I7" s="220" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="J7" s="287" t="n">
-        <v>8.08</v>
-      </c>
-      <c r="K7" s="288" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="278" t="inlineStr">
+      <c r="A8" s="212" t="inlineStr">
         <is>
           <t>BAY.BK</t>
         </is>
       </c>
-      <c r="B8" s="279" t="inlineStr">
+      <c r="B8" s="213" t="inlineStr">
         <is>
           <t>BAY</t>
         </is>
       </c>
-      <c r="C8" s="280" t="n">
+      <c r="C8" s="214" t="n">
         <v>1000</v>
       </c>
-      <c r="D8" s="281" t="n">
+      <c r="D8" s="215" t="n">
         <v>26</v>
       </c>
-      <c r="E8" s="282" t="n">
+      <c r="E8" s="216" t="n">
         <v>27.5</v>
       </c>
-      <c r="F8" s="283">
+      <c r="F8" s="217">
         <f>C8*E8</f>
         <v/>
       </c>
-      <c r="G8" s="284">
+      <c r="G8" s="218">
         <f>F8-C8*D8</f>
         <v/>
       </c>
-      <c r="H8" s="285">
+      <c r="H8" s="219">
         <f>(E8-D8)/D8</f>
         <v/>
       </c>
-      <c r="I8" s="286" t="inlineStr">
+      <c r="I8" s="220" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="J8" s="287" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="K8" s="288" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="289" t="inlineStr">
+      <c r="A9" s="221" t="inlineStr">
         <is>
           <t>CK.BK</t>
         </is>
       </c>
-      <c r="B9" s="290" t="inlineStr">
+      <c r="B9" s="222" t="inlineStr">
         <is>
           <t>CK</t>
         </is>
       </c>
-      <c r="C9" s="291" t="n">
+      <c r="C9" s="223" t="n">
         <v>1600</v>
       </c>
-      <c r="D9" s="292" t="n">
+      <c r="D9" s="224" t="n">
         <v>17.2</v>
       </c>
-      <c r="E9" s="293" t="n">
+      <c r="E9" s="225" t="n">
         <v>16.5</v>
       </c>
-      <c r="F9" s="294">
+      <c r="F9" s="226">
         <f>C9*E9</f>
         <v/>
       </c>
-      <c r="G9" s="295">
+      <c r="G9" s="227">
         <f>F9-C9*D9</f>
         <v/>
       </c>
-      <c r="H9" s="296">
+      <c r="H9" s="228">
         <f>(E9-D9)/D9</f>
         <v/>
       </c>
-      <c r="I9" s="297" t="inlineStr">
+      <c r="I9" s="229" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="J9" s="298" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="K9" s="299" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="265" t="inlineStr">
+      <c r="A10" s="203" t="inlineStr">
         <is>
           <t>AMATA.BK</t>
         </is>
       </c>
-      <c r="B10" s="266" t="inlineStr">
+      <c r="B10" s="204" t="inlineStr">
         <is>
           <t>AMATA</t>
         </is>
       </c>
-      <c r="C10" s="267" t="n">
+      <c r="C10" s="205" t="n">
         <v>1300</v>
       </c>
-      <c r="D10" s="268" t="n">
+      <c r="D10" s="206" t="n">
         <v>20.5</v>
       </c>
-      <c r="E10" s="269" t="n">
+      <c r="E10" s="207" t="n">
         <v>20.29999923706055</v>
       </c>
-      <c r="F10" s="270">
+      <c r="F10" s="208">
         <f>C10*E10</f>
         <v/>
       </c>
-      <c r="G10" s="271">
+      <c r="G10" s="209">
         <f>F10-C10*D10</f>
         <v/>
       </c>
-      <c r="H10" s="272">
+      <c r="H10" s="210">
         <f>(E10-D10)/D10</f>
         <v/>
       </c>
-      <c r="I10" s="273" t="inlineStr">
+      <c r="I10" s="211" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="J10" s="274" t="n">
-        <v>8.68</v>
-      </c>
-      <c r="K10" s="275" t="inlineStr">
-        <is>
-          <t>STRONG BUY</t>
-        </is>
-      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="265" t="inlineStr">
+      <c r="A11" s="203" t="inlineStr">
         <is>
           <t>KTC.BK</t>
         </is>
       </c>
-      <c r="B11" s="266" t="inlineStr">
+      <c r="B11" s="204" t="inlineStr">
         <is>
           <t>KTC</t>
         </is>
       </c>
-      <c r="C11" s="267" t="n">
+      <c r="C11" s="205" t="n">
         <v>900</v>
       </c>
-      <c r="D11" s="268" t="n">
+      <c r="D11" s="206" t="n">
         <v>29.25</v>
       </c>
-      <c r="E11" s="269" t="n">
+      <c r="E11" s="207" t="n">
         <v>29.25</v>
       </c>
-      <c r="F11" s="270">
+      <c r="F11" s="208">
         <f>C11*E11</f>
         <v/>
       </c>
-      <c r="G11" s="300">
+      <c r="G11" s="230">
         <f>F11-C11*D11</f>
         <v/>
       </c>
-      <c r="H11" s="301">
+      <c r="H11" s="231">
         <f>(E11-D11)/D11</f>
         <v/>
       </c>
-      <c r="I11" s="273" t="inlineStr">
+      <c r="I11" s="211" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="J11" s="274" t="n">
-        <v>7.76</v>
-      </c>
-      <c r="K11" s="275" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="265" t="inlineStr">
+      <c r="A12" s="203" t="inlineStr">
         <is>
           <t>TISCO.BK</t>
         </is>
       </c>
-      <c r="B12" s="266" t="inlineStr">
+      <c r="B12" s="204" t="inlineStr">
         <is>
           <t>TISCO</t>
         </is>
       </c>
-      <c r="C12" s="267" t="n">
+      <c r="C12" s="205" t="n">
         <v>200</v>
       </c>
-      <c r="D12" s="268" t="n">
+      <c r="D12" s="206" t="n">
         <v>113.5</v>
       </c>
-      <c r="E12" s="269" t="n">
+      <c r="E12" s="207" t="n">
         <v>113.5</v>
       </c>
-      <c r="F12" s="270">
+      <c r="F12" s="208">
         <f>C12*E12</f>
         <v/>
       </c>
-      <c r="G12" s="300">
+      <c r="G12" s="230">
         <f>F12-C12*D12</f>
         <v/>
       </c>
-      <c r="H12" s="301">
+      <c r="H12" s="231">
         <f>(E12-D12)/D12</f>
         <v/>
       </c>
-      <c r="I12" s="273" t="inlineStr">
+      <c r="I12" s="211" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="J12" s="276" t="n">
-        <v>7.16</v>
-      </c>
-      <c r="K12" s="277" t="inlineStr">
-        <is>
-          <t>WEAK</t>
-        </is>
-      </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="302" t="inlineStr">
+      <c r="B13" s="232" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F13" s="303">
+      <c r="F13" s="233">
         <f>SUM(F3:F12)</f>
         <v/>
       </c>
-      <c r="G13" s="304">
+      <c r="G13" s="234">
         <f>SUM(G3:G12)</f>
         <v/>
       </c>
-      <c r="H13" s="305">
+      <c r="H13" s="235">
         <f>G13/SUMPRODUCT(C3:C12,D3:D12)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2362,14 +2014,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="263" t="inlineStr">
-        <is>
-          <t>Today's Trades  —  27 Apr 2026</t>
+      <c r="A1" s="201" t="inlineStr">
+        <is>
+          <t>Today's Trades  —  24 Apr 2026</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="306" t="inlineStr">
+      <c r="A3" s="236" t="inlineStr">
         <is>
           <t>No trades were executed today.</t>
         </is>
@@ -2407,509 +2059,509 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="263" t="inlineStr">
+      <c r="A1" s="201" t="inlineStr">
         <is>
           <t>Complete Trade History  —  since 2026-04-21</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="264" t="inlineStr">
+      <c r="A2" s="202" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B2" s="264" t="inlineStr">
+      <c r="B2" s="202" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="C2" s="264" t="inlineStr">
+      <c r="C2" s="202" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="D2" s="264" t="inlineStr">
+      <c r="D2" s="202" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="E2" s="264" t="inlineStr">
+      <c r="E2" s="202" t="inlineStr">
         <is>
           <t>Shares</t>
         </is>
       </c>
-      <c r="F2" s="264" t="inlineStr">
+      <c r="F2" s="202" t="inlineStr">
         <is>
           <t>Price (฿)</t>
         </is>
       </c>
-      <c r="G2" s="264" t="inlineStr">
+      <c r="G2" s="202" t="inlineStr">
         <is>
           <t>Lots</t>
         </is>
       </c>
-      <c r="H2" s="264" t="inlineStr">
+      <c r="H2" s="202" t="inlineStr">
         <is>
           <t>Value (฿)</t>
         </is>
       </c>
-      <c r="I2" s="264" t="inlineStr">
+      <c r="I2" s="202" t="inlineStr">
         <is>
           <t>Realised P&amp;L (฿)</t>
         </is>
       </c>
-      <c r="J2" s="264" t="inlineStr">
+      <c r="J2" s="202" t="inlineStr">
         <is>
           <t>Reason / Signal</t>
         </is>
       </c>
     </row>
     <row r="3" ht="17" customHeight="1">
-      <c r="A3" s="307" t="inlineStr">
+      <c r="A3" s="237" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B3" s="308" t="inlineStr">
+      <c r="B3" s="238" t="inlineStr">
         <is>
           <t>TISCO.BK</t>
         </is>
       </c>
-      <c r="C3" s="309" t="inlineStr">
+      <c r="C3" s="239" t="inlineStr">
         <is>
           <t>TISCO</t>
         </is>
       </c>
-      <c r="D3" s="310" t="inlineStr">
+      <c r="D3" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E3" s="311" t="n">
+      <c r="E3" s="241" t="n">
         <v>200</v>
       </c>
-      <c r="F3" s="312" t="n">
+      <c r="F3" s="242" t="n">
         <v>113.5</v>
       </c>
-      <c r="G3" s="311" t="n">
+      <c r="G3" s="241" t="n">
         <v>2</v>
       </c>
-      <c r="H3" s="313">
+      <c r="H3" s="243">
         <f>E3*F3</f>
         <v/>
       </c>
-      <c r="I3" s="314" t="inlineStr">
+      <c r="I3" s="244" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J3" s="315" t="inlineStr">
+      <c r="J3" s="245" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="17" customHeight="1">
-      <c r="A4" s="316" t="inlineStr">
+      <c r="A4" s="246" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B4" s="317" t="inlineStr">
+      <c r="B4" s="247" t="inlineStr">
         <is>
           <t>SIRI.BK</t>
         </is>
       </c>
-      <c r="C4" s="266" t="inlineStr">
+      <c r="C4" s="204" t="inlineStr">
         <is>
           <t>SIRI</t>
         </is>
       </c>
-      <c r="D4" s="310" t="inlineStr">
+      <c r="D4" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E4" s="267" t="n">
+      <c r="E4" s="205" t="n">
         <v>20200</v>
       </c>
-      <c r="F4" s="268" t="n">
+      <c r="F4" s="206" t="n">
         <v>1.41</v>
       </c>
-      <c r="G4" s="267" t="n">
+      <c r="G4" s="205" t="n">
         <v>202</v>
       </c>
-      <c r="H4" s="270">
+      <c r="H4" s="208">
         <f>E4*F4</f>
         <v/>
       </c>
-      <c r="I4" s="318" t="inlineStr">
+      <c r="I4" s="248" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J4" s="319" t="inlineStr">
+      <c r="J4" s="249" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="307" t="inlineStr">
+      <c r="A5" s="237" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B5" s="308" t="inlineStr">
+      <c r="B5" s="238" t="inlineStr">
         <is>
           <t>TU.BK</t>
         </is>
       </c>
-      <c r="C5" s="309" t="inlineStr">
+      <c r="C5" s="239" t="inlineStr">
         <is>
           <t>TU</t>
         </is>
       </c>
-      <c r="D5" s="310" t="inlineStr">
+      <c r="D5" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E5" s="311" t="n">
+      <c r="E5" s="241" t="n">
         <v>2500</v>
       </c>
-      <c r="F5" s="312" t="n">
+      <c r="F5" s="242" t="n">
         <v>11.4</v>
       </c>
-      <c r="G5" s="311" t="n">
+      <c r="G5" s="241" t="n">
         <v>25</v>
       </c>
-      <c r="H5" s="313">
+      <c r="H5" s="243">
         <f>E5*F5</f>
         <v/>
       </c>
-      <c r="I5" s="314" t="inlineStr">
+      <c r="I5" s="244" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J5" s="315" t="inlineStr">
+      <c r="J5" s="245" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="316" t="inlineStr">
+      <c r="A6" s="246" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B6" s="317" t="inlineStr">
+      <c r="B6" s="247" t="inlineStr">
         <is>
           <t>BAY.BK</t>
         </is>
       </c>
-      <c r="C6" s="266" t="inlineStr">
+      <c r="C6" s="204" t="inlineStr">
         <is>
           <t>BAY</t>
         </is>
       </c>
-      <c r="D6" s="310" t="inlineStr">
+      <c r="D6" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E6" s="267" t="n">
+      <c r="E6" s="205" t="n">
         <v>1000</v>
       </c>
-      <c r="F6" s="268" t="n">
+      <c r="F6" s="206" t="n">
         <v>26</v>
       </c>
-      <c r="G6" s="267" t="n">
+      <c r="G6" s="205" t="n">
         <v>10</v>
       </c>
-      <c r="H6" s="270">
+      <c r="H6" s="208">
         <f>E6*F6</f>
         <v/>
       </c>
-      <c r="I6" s="318" t="inlineStr">
+      <c r="I6" s="248" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J6" s="319" t="inlineStr">
+      <c r="J6" s="249" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="307" t="inlineStr">
+      <c r="A7" s="237" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B7" s="308" t="inlineStr">
+      <c r="B7" s="238" t="inlineStr">
         <is>
           <t>KTC.BK</t>
         </is>
       </c>
-      <c r="C7" s="309" t="inlineStr">
+      <c r="C7" s="239" t="inlineStr">
         <is>
           <t>KTC</t>
         </is>
       </c>
-      <c r="D7" s="310" t="inlineStr">
+      <c r="D7" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E7" s="311" t="n">
+      <c r="E7" s="241" t="n">
         <v>900</v>
       </c>
-      <c r="F7" s="312" t="n">
+      <c r="F7" s="242" t="n">
         <v>29.25</v>
       </c>
-      <c r="G7" s="311" t="n">
+      <c r="G7" s="241" t="n">
         <v>9</v>
       </c>
-      <c r="H7" s="313">
+      <c r="H7" s="243">
         <f>E7*F7</f>
         <v/>
       </c>
-      <c r="I7" s="314" t="inlineStr">
+      <c r="I7" s="244" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J7" s="315" t="inlineStr">
+      <c r="J7" s="245" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="316" t="inlineStr">
+      <c r="A8" s="246" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B8" s="317" t="inlineStr">
+      <c r="B8" s="247" t="inlineStr">
         <is>
           <t>TQM.BK</t>
         </is>
       </c>
-      <c r="C8" s="266" t="inlineStr">
+      <c r="C8" s="204" t="inlineStr">
         <is>
           <t>TQM</t>
         </is>
       </c>
-      <c r="D8" s="310" t="inlineStr">
+      <c r="D8" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E8" s="267" t="n">
+      <c r="E8" s="205" t="n">
         <v>2000</v>
       </c>
-      <c r="F8" s="268" t="n">
+      <c r="F8" s="206" t="n">
         <v>13.7</v>
       </c>
-      <c r="G8" s="267" t="n">
+      <c r="G8" s="205" t="n">
         <v>20</v>
       </c>
-      <c r="H8" s="270">
+      <c r="H8" s="208">
         <f>E8*F8</f>
         <v/>
       </c>
-      <c r="I8" s="318" t="inlineStr">
+      <c r="I8" s="248" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J8" s="319" t="inlineStr">
+      <c r="J8" s="249" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="307" t="inlineStr">
+      <c r="A9" s="237" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B9" s="308" t="inlineStr">
+      <c r="B9" s="238" t="inlineStr">
         <is>
           <t>WHA.BK</t>
         </is>
       </c>
-      <c r="C9" s="309" t="inlineStr">
+      <c r="C9" s="239" t="inlineStr">
         <is>
           <t>WHA</t>
         </is>
       </c>
-      <c r="D9" s="310" t="inlineStr">
+      <c r="D9" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E9" s="311" t="n">
+      <c r="E9" s="241" t="n">
         <v>6400</v>
       </c>
-      <c r="F9" s="312" t="n">
+      <c r="F9" s="242" t="n">
         <v>4.4</v>
       </c>
-      <c r="G9" s="311" t="n">
+      <c r="G9" s="241" t="n">
         <v>64</v>
       </c>
-      <c r="H9" s="313">
+      <c r="H9" s="243">
         <f>E9*F9</f>
         <v/>
       </c>
-      <c r="I9" s="314" t="inlineStr">
+      <c r="I9" s="244" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J9" s="315" t="inlineStr">
+      <c r="J9" s="245" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="316" t="inlineStr">
+      <c r="A10" s="246" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B10" s="317" t="inlineStr">
+      <c r="B10" s="247" t="inlineStr">
         <is>
           <t>JASIF.BK</t>
         </is>
       </c>
-      <c r="C10" s="266" t="inlineStr">
+      <c r="C10" s="204" t="inlineStr">
         <is>
           <t>JASIF</t>
         </is>
       </c>
-      <c r="D10" s="310" t="inlineStr">
+      <c r="D10" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E10" s="267" t="n">
+      <c r="E10" s="205" t="n">
         <v>4200</v>
       </c>
-      <c r="F10" s="268" t="n">
+      <c r="F10" s="206" t="n">
         <v>6.7</v>
       </c>
-      <c r="G10" s="267" t="n">
+      <c r="G10" s="205" t="n">
         <v>42</v>
       </c>
-      <c r="H10" s="270">
+      <c r="H10" s="208">
         <f>E10*F10</f>
         <v/>
       </c>
-      <c r="I10" s="318" t="inlineStr">
+      <c r="I10" s="248" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J10" s="319" t="inlineStr">
+      <c r="J10" s="249" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="307" t="inlineStr">
+      <c r="A11" s="237" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B11" s="308" t="inlineStr">
+      <c r="B11" s="238" t="inlineStr">
         <is>
           <t>CK.BK</t>
         </is>
       </c>
-      <c r="C11" s="309" t="inlineStr">
+      <c r="C11" s="239" t="inlineStr">
         <is>
           <t>CK</t>
         </is>
       </c>
-      <c r="D11" s="310" t="inlineStr">
+      <c r="D11" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E11" s="311" t="n">
+      <c r="E11" s="241" t="n">
         <v>1600</v>
       </c>
-      <c r="F11" s="312" t="n">
+      <c r="F11" s="242" t="n">
         <v>17.2</v>
       </c>
-      <c r="G11" s="311" t="n">
+      <c r="G11" s="241" t="n">
         <v>16</v>
       </c>
-      <c r="H11" s="313">
+      <c r="H11" s="243">
         <f>E11*F11</f>
         <v/>
       </c>
-      <c r="I11" s="314" t="inlineStr">
+      <c r="I11" s="244" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J11" s="315" t="inlineStr">
+      <c r="J11" s="245" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="316" t="inlineStr">
+      <c r="A12" s="246" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="B12" s="317" t="inlineStr">
+      <c r="B12" s="247" t="inlineStr">
         <is>
           <t>AMATA.BK</t>
         </is>
       </c>
-      <c r="C12" s="266" t="inlineStr">
+      <c r="C12" s="204" t="inlineStr">
         <is>
           <t>AMATA</t>
         </is>
       </c>
-      <c r="D12" s="310" t="inlineStr">
+      <c r="D12" s="240" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="E12" s="267" t="n">
+      <c r="E12" s="205" t="n">
         <v>1300</v>
       </c>
-      <c r="F12" s="268" t="n">
+      <c r="F12" s="206" t="n">
         <v>20.5</v>
       </c>
-      <c r="G12" s="267" t="n">
+      <c r="G12" s="205" t="n">
         <v>13</v>
       </c>
-      <c r="H12" s="270">
+      <c r="H12" s="208">
         <f>E12*F12</f>
         <v/>
       </c>
-      <c r="I12" s="318" t="inlineStr">
+      <c r="I12" s="248" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J12" s="319" t="inlineStr">
+      <c r="J12" s="249" t="inlineStr">
         <is>
           <t>BUY (Day 1)</t>
         </is>
@@ -2921,11 +2573,11 @@
           <t>TOTAL TRADES</t>
         </is>
       </c>
-      <c r="H14" s="320">
+      <c r="H14" s="250">
         <f>SUM(H3:H12)</f>
         <v/>
       </c>
-      <c r="I14" s="320">
+      <c r="I14" s="250">
         <f>SUM(I3:I12)</f>
         <v/>
       </c>

</xml_diff>